<commit_message>
Add October budget explanation and email draft
Co-authored-by: peterli0913 <peterli0913@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/2026/PP-2610 Monthly Budget Application Form_.xlsx
+++ b/2026/PP-2610 Monthly Budget Application Form_.xlsx
@@ -5350,7 +5350,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -5439,12 +5439,12 @@
         <v>0</v>
       </c>
       <c r="E4" s="136">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B4,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
-        <v>9000</v>
+        <f>SUMPRODUCT(('K(Cost center)-Opex (Service)'!$D$4:$D$40=$B4)*('K(Cost center)-Opex (Service)'!$X$4:$X$40=E$3)*('K(Cost center)-Opex (Service)'!$N$4:$N$40)*IF(ISNUMBER('K(Cost center)-Opex (Service)'!$O$4:$O$40),'K(Cost center)-Opex (Service)'!$O$4:$O$40,0))+SUMPRODUCT(('K(Cost center)-Opex (Service)'!$D$4:$D$40=$B4)*('K(Cost center)-Opex (Service)'!$X$4:$X$40=E$3)*(NOT(ISNUMBER('K(Cost center)-Opex (Service)'!$O$4:$O$40)))*('K(Cost center)-Opex (Service)'!$S$4:$S$40))</f>
+        <v>7500</v>
       </c>
       <c r="F4" s="136">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B4,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
-        <v>20368</v>
+        <f>SUMPRODUCT(('K(Cost center)-Opex (Service)'!$D$4:$D$40=$B4)*('K(Cost center)-Opex (Service)'!$X$4:$X$40=F$3)*('K(Cost center)-Opex (Service)'!$N$4:$N$40)*IF(ISNUMBER('K(Cost center)-Opex (Service)'!$O$4:$O$40),'K(Cost center)-Opex (Service)'!$O$4:$O$40,0))</f>
+        <v>16973</v>
       </c>
       <c r="G4" s="136">
         <f t="shared" ref="G4:G10" si="0">SUM(C4:D4)</f>
@@ -5452,7 +5452,7 @@
       </c>
       <c r="H4" s="146">
         <f t="shared" ref="H4:H10" si="1">SUM(E4:F4)</f>
-        <v>29368</v>
+        <v>24473</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15.75" customHeight="1">
@@ -5469,12 +5469,12 @@
         <v>0</v>
       </c>
       <c r="E5" s="136">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B5,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <f>SUMPRODUCT(('K(Cost center)-Opex (Service)'!$D$4:$D$40=$B5)*('K(Cost center)-Opex (Service)'!$X$4:$X$40=E$3)*('K(Cost center)-Opex (Service)'!$N$4:$N$40)*IF(ISNUMBER('K(Cost center)-Opex (Service)'!$O$4:$O$40),'K(Cost center)-Opex (Service)'!$O$4:$O$40,0))+SUMPRODUCT(('K(Cost center)-Opex (Service)'!$D$4:$D$40=$B5)*('K(Cost center)-Opex (Service)'!$X$4:$X$40=E$3)*(NOT(ISNUMBER('K(Cost center)-Opex (Service)'!$O$4:$O$40)))*('K(Cost center)-Opex (Service)'!$S$4:$S$40))</f>
         <v>0</v>
       </c>
       <c r="F5" s="136">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B5,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
-        <v>1200</v>
+        <f>SUMPRODUCT(('K(Cost center)-Opex (Service)'!$D$4:$D$40=$B5)*('K(Cost center)-Opex (Service)'!$X$4:$X$40=F$3)*('K(Cost center)-Opex (Service)'!$N$4:$N$40)*IF(ISNUMBER('K(Cost center)-Opex (Service)'!$O$4:$O$40),'K(Cost center)-Opex (Service)'!$O$4:$O$40,0))</f>
+        <v>1000</v>
       </c>
       <c r="G5" s="136">
         <f t="shared" si="0"/>
@@ -5482,7 +5482,7 @@
       </c>
       <c r="H5" s="146">
         <f t="shared" si="1"/>
-        <v>1200</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15.75" customHeight="1">
@@ -5499,11 +5499,11 @@
         <v>0</v>
       </c>
       <c r="E6" s="136">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B6,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <f>SUMPRODUCT(('K(Cost center)-Opex (Service)'!$D$4:$D$40=$B6)*('K(Cost center)-Opex (Service)'!$X$4:$X$40=E$3)*('K(Cost center)-Opex (Service)'!$N$4:$N$40)*IF(ISNUMBER('K(Cost center)-Opex (Service)'!$O$4:$O$40),'K(Cost center)-Opex (Service)'!$O$4:$O$40,0))+SUMPRODUCT(('K(Cost center)-Opex (Service)'!$D$4:$D$40=$B6)*('K(Cost center)-Opex (Service)'!$X$4:$X$40=E$3)*(NOT(ISNUMBER('K(Cost center)-Opex (Service)'!$O$4:$O$40)))*('K(Cost center)-Opex (Service)'!$S$4:$S$40))</f>
         <v>0</v>
       </c>
       <c r="F6" s="136">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B6,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
+        <f>SUMPRODUCT(('K(Cost center)-Opex (Service)'!$D$4:$D$40=$B6)*('K(Cost center)-Opex (Service)'!$X$4:$X$40=F$3)*('K(Cost center)-Opex (Service)'!$N$4:$N$40)*IF(ISNUMBER('K(Cost center)-Opex (Service)'!$O$4:$O$40),'K(Cost center)-Opex (Service)'!$O$4:$O$40,0))</f>
         <v>0</v>
       </c>
       <c r="G6" s="136">
@@ -5529,12 +5529,12 @@
         <v>0</v>
       </c>
       <c r="E7" s="136">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B7,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <f>SUMPRODUCT(('K(Cost center)-Opex (Service)'!$D$4:$D$40=$B7)*('K(Cost center)-Opex (Service)'!$X$4:$X$40=E$3)*('K(Cost center)-Opex (Service)'!$N$4:$N$40)*IF(ISNUMBER('K(Cost center)-Opex (Service)'!$O$4:$O$40),'K(Cost center)-Opex (Service)'!$O$4:$O$40,0))+SUMPRODUCT(('K(Cost center)-Opex (Service)'!$D$4:$D$40=$B7)*('K(Cost center)-Opex (Service)'!$X$4:$X$40=E$3)*(NOT(ISNUMBER('K(Cost center)-Opex (Service)'!$O$4:$O$40)))*('K(Cost center)-Opex (Service)'!$S$4:$S$40))</f>
         <v>0</v>
       </c>
       <c r="F7" s="136">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B7,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
-        <v>1560</v>
+        <f>SUMPRODUCT(('K(Cost center)-Opex (Service)'!$D$4:$D$40=$B7)*('K(Cost center)-Opex (Service)'!$X$4:$X$40=F$3)*('K(Cost center)-Opex (Service)'!$N$4:$N$40)*IF(ISNUMBER('K(Cost center)-Opex (Service)'!$O$4:$O$40),'K(Cost center)-Opex (Service)'!$O$4:$O$40,0))</f>
+        <v>1300</v>
       </c>
       <c r="G7" s="136">
         <f t="shared" si="0"/>
@@ -5542,7 +5542,7 @@
       </c>
       <c r="H7" s="146">
         <f t="shared" si="1"/>
-        <v>1560</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15.75" customHeight="1">
@@ -5559,11 +5559,11 @@
         <v>0</v>
       </c>
       <c r="E8" s="136">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B8,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <f>SUMPRODUCT(('K(Cost center)-Opex (Service)'!$D$4:$D$40=$B8)*('K(Cost center)-Opex (Service)'!$X$4:$X$40=E$3)*('K(Cost center)-Opex (Service)'!$N$4:$N$40)*IF(ISNUMBER('K(Cost center)-Opex (Service)'!$O$4:$O$40),'K(Cost center)-Opex (Service)'!$O$4:$O$40,0))+SUMPRODUCT(('K(Cost center)-Opex (Service)'!$D$4:$D$40=$B8)*('K(Cost center)-Opex (Service)'!$X$4:$X$40=E$3)*(NOT(ISNUMBER('K(Cost center)-Opex (Service)'!$O$4:$O$40)))*('K(Cost center)-Opex (Service)'!$S$4:$S$40))</f>
         <v>0</v>
       </c>
       <c r="F8" s="136">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B8,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
+        <f>SUMPRODUCT(('K(Cost center)-Opex (Service)'!$D$4:$D$40=$B8)*('K(Cost center)-Opex (Service)'!$X$4:$X$40=F$3)*('K(Cost center)-Opex (Service)'!$N$4:$N$40)*IF(ISNUMBER('K(Cost center)-Opex (Service)'!$O$4:$O$40),'K(Cost center)-Opex (Service)'!$O$4:$O$40,0))</f>
         <v>0</v>
       </c>
       <c r="G8" s="136">
@@ -5589,11 +5589,11 @@
         <v>0</v>
       </c>
       <c r="E9" s="136">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B9,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
-        <v>24000</v>
+        <f>SUMPRODUCT(('K(Cost center)-Opex (Service)'!$D$4:$D$40=$B9)*('K(Cost center)-Opex (Service)'!$X$4:$X$40=E$3)*('K(Cost center)-Opex (Service)'!$N$4:$N$40)*IF(ISNUMBER('K(Cost center)-Opex (Service)'!$O$4:$O$40),'K(Cost center)-Opex (Service)'!$O$4:$O$40,0))+SUMPRODUCT(('K(Cost center)-Opex (Service)'!$D$4:$D$40=$B9)*('K(Cost center)-Opex (Service)'!$X$4:$X$40=E$3)*(NOT(ISNUMBER('K(Cost center)-Opex (Service)'!$O$4:$O$40)))*('K(Cost center)-Opex (Service)'!$S$4:$S$40))</f>
+        <v>20000</v>
       </c>
       <c r="F9" s="136">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B9,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
+        <f>SUMPRODUCT(('K(Cost center)-Opex (Service)'!$D$4:$D$40=$B9)*('K(Cost center)-Opex (Service)'!$X$4:$X$40=F$3)*('K(Cost center)-Opex (Service)'!$N$4:$N$40)*IF(ISNUMBER('K(Cost center)-Opex (Service)'!$O$4:$O$40),'K(Cost center)-Opex (Service)'!$O$4:$O$40,0))</f>
         <v>0</v>
       </c>
       <c r="G9" s="136">
@@ -5602,7 +5602,7 @@
       </c>
       <c r="H9" s="146">
         <f t="shared" si="1"/>
-        <v>24000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15.75" customHeight="1">
@@ -5619,11 +5619,11 @@
         <v>0</v>
       </c>
       <c r="E10" s="136">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B10,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <f>SUMPRODUCT(('K(Cost center)-Opex (Service)'!$D$4:$D$40=$B10)*('K(Cost center)-Opex (Service)'!$X$4:$X$40=E$3)*('K(Cost center)-Opex (Service)'!$N$4:$N$40)*IF(ISNUMBER('K(Cost center)-Opex (Service)'!$O$4:$O$40),'K(Cost center)-Opex (Service)'!$O$4:$O$40,0))+SUMPRODUCT(('K(Cost center)-Opex (Service)'!$D$4:$D$40=$B10)*('K(Cost center)-Opex (Service)'!$X$4:$X$40=E$3)*(NOT(ISNUMBER('K(Cost center)-Opex (Service)'!$O$4:$O$40)))*('K(Cost center)-Opex (Service)'!$S$4:$S$40))</f>
         <v>38184</v>
       </c>
       <c r="F10" s="136">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B10,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
+        <f>SUMPRODUCT(('K(Cost center)-Opex (Service)'!$D$4:$D$40=$B10)*('K(Cost center)-Opex (Service)'!$X$4:$X$40=F$3)*('K(Cost center)-Opex (Service)'!$N$4:$N$40)*IF(ISNUMBER('K(Cost center)-Opex (Service)'!$O$4:$O$40),'K(Cost center)-Opex (Service)'!$O$4:$O$40,0))</f>
         <v>0</v>
       </c>
       <c r="G10" s="136">
@@ -5650,11 +5650,11 @@
       </c>
       <c r="E11" s="144">
         <f t="shared" si="2"/>
-        <v>71184</v>
+        <v>65684</v>
       </c>
       <c r="F11" s="144">
         <f t="shared" si="2"/>
-        <v>23128</v>
+        <v>19273</v>
       </c>
       <c r="G11" s="143">
         <f t="shared" si="2"/>
@@ -5662,7 +5662,7 @@
       </c>
       <c r="H11" s="147">
         <f t="shared" si="2"/>
-        <v>94312</v>
+        <v>84957</v>
       </c>
     </row>
   </sheetData>

</xml_diff>